<commit_message>
Add baseline QC Excel review export
Ultraworked with [Sisyphus](https://github.com/code-yeongyu/oh-my-openagent)

Co-authored-by: Sisyphus <clio-agent@sisyphuslabs.ai>
</commit_message>
<xml_diff>
--- a/data/reference/datasets.xlsx
+++ b/data/reference/datasets.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28260" windowHeight="12420"/>
+    <workbookView windowWidth="28260" windowHeight="12680"/>
   </bookViews>
   <sheets>
     <sheet name="pbmc_samples" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">pbmc_samples!$A$1:$G$323</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">pbmc_samples!$A$1:$G$365</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2261" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2555" uniqueCount="498">
   <si>
     <t>样本名(GSM*)</t>
   </si>
@@ -1103,16 +1103,259 @@
     <t>GSM5737278</t>
   </si>
   <si>
+    <t>GSM8671412</t>
+  </si>
+  <si>
+    <t>GSE283744</t>
+  </si>
+  <si>
+    <t>9.5月</t>
+  </si>
+  <si>
+    <t>fragment</t>
+  </si>
+  <si>
+    <t>COVID-19</t>
+  </si>
+  <si>
+    <t>GSM8671413</t>
+  </si>
+  <si>
+    <t>1月</t>
+  </si>
+  <si>
+    <t>GSM8671414</t>
+  </si>
+  <si>
+    <t>7.5月</t>
+  </si>
+  <si>
+    <t>GSM8671415</t>
+  </si>
+  <si>
+    <t>0.5月</t>
+  </si>
+  <si>
+    <t>GSM8671416</t>
+  </si>
+  <si>
+    <t>6.4月</t>
+  </si>
+  <si>
+    <t>GSM8671417</t>
+  </si>
+  <si>
+    <t>1.2月</t>
+  </si>
+  <si>
+    <t>GSM8671418</t>
+  </si>
+  <si>
+    <t>6.63月</t>
+  </si>
+  <si>
+    <t>GSM8671419</t>
+  </si>
+  <si>
+    <t>19.2月</t>
+  </si>
+  <si>
+    <t>GSM8671420</t>
+  </si>
+  <si>
+    <t>27.5月</t>
+  </si>
+  <si>
+    <t>GSM8671421</t>
+  </si>
+  <si>
+    <t>0.6月</t>
+  </si>
+  <si>
+    <t>GSM8671422</t>
+  </si>
+  <si>
+    <t>7.86月</t>
+  </si>
+  <si>
+    <t>GSM8671423</t>
+  </si>
+  <si>
+    <t>0.13月</t>
+  </si>
+  <si>
+    <t>GSM8671424</t>
+  </si>
+  <si>
+    <t>11.8月</t>
+  </si>
+  <si>
+    <t>GSM8671425</t>
+  </si>
+  <si>
+    <t>GSM8671426</t>
+  </si>
+  <si>
+    <t>0.86月</t>
+  </si>
+  <si>
+    <t>GSM8671427</t>
+  </si>
+  <si>
+    <t>0.96月</t>
+  </si>
+  <si>
+    <t>GSM8671428</t>
+  </si>
+  <si>
+    <t>2月</t>
+  </si>
+  <si>
+    <t>GSM8671429</t>
+  </si>
+  <si>
+    <t>1.9月</t>
+  </si>
+  <si>
+    <t>GSM8671430</t>
+  </si>
+  <si>
+    <t>0.76月</t>
+  </si>
+  <si>
+    <t>GSM8671431</t>
+  </si>
+  <si>
+    <t>1.3月</t>
+  </si>
+  <si>
+    <t>GSM8671432</t>
+  </si>
+  <si>
+    <t>GSM8671433</t>
+  </si>
+  <si>
+    <t>14月</t>
+  </si>
+  <si>
+    <t>GSM8671434</t>
+  </si>
+  <si>
+    <t>1.4月</t>
+  </si>
+  <si>
+    <t>GSM8671435</t>
+  </si>
+  <si>
+    <t>3.1月</t>
+  </si>
+  <si>
+    <t>GSM8671436</t>
+  </si>
+  <si>
+    <t>13月</t>
+  </si>
+  <si>
+    <t>GSM8671437</t>
+  </si>
+  <si>
+    <t>1.47月</t>
+  </si>
+  <si>
+    <t>RSV</t>
+  </si>
+  <si>
+    <t>GSM8671438</t>
+  </si>
+  <si>
+    <t>GSM8671439</t>
+  </si>
+  <si>
+    <t>12.8月</t>
+  </si>
+  <si>
+    <t>GSM8671440</t>
+  </si>
+  <si>
+    <t>2.4月</t>
+  </si>
+  <si>
+    <t>GSM8671441</t>
+  </si>
+  <si>
+    <t>0.8月</t>
+  </si>
+  <si>
+    <t>GSM8671442</t>
+  </si>
+  <si>
+    <t>2.8月</t>
+  </si>
+  <si>
+    <t>GSM8671443</t>
+  </si>
+  <si>
+    <t>13.7月</t>
+  </si>
+  <si>
+    <t>GSM8671444</t>
+  </si>
+  <si>
+    <t>5.37月</t>
+  </si>
+  <si>
+    <t>GSM8671445</t>
+  </si>
+  <si>
+    <t>GSM8671446</t>
+  </si>
+  <si>
+    <t>10.5月</t>
+  </si>
+  <si>
+    <t>GSM8671447</t>
+  </si>
+  <si>
+    <t>1.1月</t>
+  </si>
+  <si>
+    <t>GSM8671448</t>
+  </si>
+  <si>
+    <t>4.3月</t>
+  </si>
+  <si>
+    <t>GSM8671449</t>
+  </si>
+  <si>
+    <t>1.6月</t>
+  </si>
+  <si>
+    <t>GSM8671450</t>
+  </si>
+  <si>
+    <t>4.2月</t>
+  </si>
+  <si>
+    <t>GSM8671451</t>
+  </si>
+  <si>
+    <t>3.8月</t>
+  </si>
+  <si>
+    <t>GSM8671452</t>
+  </si>
+  <si>
+    <t>GSM8671453</t>
+  </si>
+  <si>
+    <t>6.2月</t>
+  </si>
+  <si>
     <t>GSM8671454</t>
   </si>
   <si>
-    <t>GSE283744</t>
-  </si>
-  <si>
     <t>1.92月</t>
-  </si>
-  <si>
-    <t>fragment</t>
   </si>
   <si>
     <t>GSM8671455</t>
@@ -1137,15 +1380,9 @@
     <t>GSM8671458</t>
   </si>
   <si>
-    <t>1.6月</t>
-  </si>
-  <si>
     <t>GSM8671459</t>
   </si>
   <si>
-    <t>1.9月</t>
-  </si>
-  <si>
     <t>GSM8671460</t>
   </si>
   <si>
@@ -1153,9 +1390,6 @@
   </si>
   <si>
     <t>GSM8671461</t>
-  </si>
-  <si>
-    <t>0.5月</t>
   </si>
   <si>
     <t>GSM8671462</t>
@@ -1303,7 +1537,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1325,6 +1559,13 @@
       <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1796,128 +2037,128 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1928,7 +2169,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
@@ -1937,7 +2181,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2284,7 +2528,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G324"/>
+  <dimension ref="A1:G366"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="17.125" customWidth="1"/>
@@ -8708,13 +8952,13 @@
       <c r="F279" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G279" s="1" t="s">
-        <v>13</v>
+      <c r="G279" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="280" spans="1:7">
       <c r="A280" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B280" s="1" t="s">
         <v>358</v>
@@ -8726,18 +8970,18 @@
         <v>10</v>
       </c>
       <c r="E280" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F280" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G280" s="1" t="s">
-        <v>13</v>
+      <c r="G280" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="281" spans="1:7">
       <c r="A281" s="1" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B281" s="1" t="s">
         <v>358</v>
@@ -8749,18 +8993,18 @@
         <v>10</v>
       </c>
       <c r="E281" s="1" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F281" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G281" s="1" t="s">
-        <v>13</v>
+      <c r="G281" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="282" spans="1:7">
       <c r="A282" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B282" s="1" t="s">
         <v>358</v>
@@ -8772,18 +9016,18 @@
         <v>10</v>
       </c>
       <c r="E282" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F282" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G282" s="1" t="s">
-        <v>13</v>
+      <c r="G282" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="283" spans="1:7">
       <c r="A283" s="1" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B283" s="1" t="s">
         <v>358</v>
@@ -8795,18 +9039,18 @@
         <v>10</v>
       </c>
       <c r="E283" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F283" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G283" s="1" t="s">
-        <v>13</v>
+      <c r="G283" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="284" spans="1:7">
       <c r="A284" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B284" s="1" t="s">
         <v>358</v>
@@ -8818,18 +9062,18 @@
         <v>10</v>
       </c>
       <c r="E284" s="1" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F284" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G284" s="1" t="s">
-        <v>13</v>
+      <c r="G284" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="285" spans="1:7">
       <c r="A285" s="1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B285" s="1" t="s">
         <v>358</v>
@@ -8841,18 +9085,18 @@
         <v>10</v>
       </c>
       <c r="E285" s="1" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F285" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G285" s="1" t="s">
-        <v>13</v>
+      <c r="G285" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="286" spans="1:7">
       <c r="A286" s="1" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B286" s="1" t="s">
         <v>358</v>
@@ -8864,18 +9108,18 @@
         <v>10</v>
       </c>
       <c r="E286" s="1" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F286" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G286" s="1" t="s">
-        <v>13</v>
+      <c r="G286" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="287" spans="1:7">
       <c r="A287" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B287" s="1" t="s">
         <v>358</v>
@@ -8887,18 +9131,18 @@
         <v>10</v>
       </c>
       <c r="E287" s="1" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F287" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G287" s="1" t="s">
-        <v>13</v>
+      <c r="G287" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="288" spans="1:7">
       <c r="A288" s="1" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B288" s="1" t="s">
         <v>358</v>
@@ -8910,21 +9154,21 @@
         <v>10</v>
       </c>
       <c r="E288" s="1" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F288" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G288" s="1" t="s">
-        <v>13</v>
+      <c r="G288" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="289" spans="1:7">
       <c r="A289" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C289" s="1" t="s">
         <v>74</v>
@@ -8933,21 +9177,21 @@
         <v>10</v>
       </c>
       <c r="E289" s="1" t="s">
-        <v>332</v>
+        <v>381</v>
       </c>
       <c r="F289" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G289" s="1" t="s">
-        <v>13</v>
+      <c r="G289" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="290" spans="1:7">
       <c r="A290" s="1" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B290" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C290" s="1" t="s">
         <v>74</v>
@@ -8956,21 +9200,21 @@
         <v>10</v>
       </c>
       <c r="E290" s="1" t="s">
-        <v>332</v>
+        <v>383</v>
       </c>
       <c r="F290" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G290" s="1" t="s">
-        <v>13</v>
+      <c r="G290" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="291" spans="1:7">
       <c r="A291" s="1" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B291" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C291" s="1" t="s">
         <v>74</v>
@@ -8979,21 +9223,21 @@
         <v>10</v>
       </c>
       <c r="E291" s="1" t="s">
-        <v>332</v>
+        <v>385</v>
       </c>
       <c r="F291" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G291" s="1" t="s">
-        <v>13</v>
+      <c r="G291" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="292" spans="1:7">
       <c r="A292" s="1" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="B292" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C292" s="1" t="s">
         <v>74</v>
@@ -9002,21 +9246,21 @@
         <v>10</v>
       </c>
       <c r="E292" s="1" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
       <c r="F292" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G292" s="1" t="s">
-        <v>13</v>
+      <c r="G292" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="293" spans="1:7">
       <c r="A293" s="1" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="B293" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C293" s="1" t="s">
         <v>74</v>
@@ -9025,21 +9269,21 @@
         <v>10</v>
       </c>
       <c r="E293" s="1" t="s">
-        <v>332</v>
+        <v>388</v>
       </c>
       <c r="F293" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G293" s="1" t="s">
-        <v>13</v>
+      <c r="G293" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="294" spans="1:7">
       <c r="A294" s="1" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="B294" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C294" s="1" t="s">
         <v>74</v>
@@ -9048,21 +9292,21 @@
         <v>10</v>
       </c>
       <c r="E294" s="1" t="s">
-        <v>332</v>
+        <v>390</v>
       </c>
       <c r="F294" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G294" s="1" t="s">
-        <v>13</v>
+      <c r="G294" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="295" spans="1:7">
       <c r="A295" s="1" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="B295" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C295" s="1" t="s">
         <v>74</v>
@@ -9071,21 +9315,21 @@
         <v>10</v>
       </c>
       <c r="E295" s="1" t="s">
-        <v>332</v>
+        <v>392</v>
       </c>
       <c r="F295" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G295" s="1" t="s">
-        <v>13</v>
+      <c r="G295" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="296" spans="1:7">
       <c r="A296" s="1" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="B296" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C296" s="1" t="s">
         <v>74</v>
@@ -9094,21 +9338,21 @@
         <v>10</v>
       </c>
       <c r="E296" s="1" t="s">
-        <v>332</v>
+        <v>394</v>
       </c>
       <c r="F296" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G296" s="1" t="s">
-        <v>13</v>
+      <c r="G296" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="297" spans="1:7">
       <c r="A297" s="1" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="B297" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C297" s="1" t="s">
         <v>74</v>
@@ -9117,21 +9361,21 @@
         <v>10</v>
       </c>
       <c r="E297" s="1" t="s">
-        <v>332</v>
+        <v>396</v>
       </c>
       <c r="F297" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G297" s="1" t="s">
-        <v>13</v>
+      <c r="G297" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="298" spans="1:7">
       <c r="A298" s="1" t="s">
-        <v>388</v>
+        <v>397</v>
       </c>
       <c r="B298" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C298" s="1" t="s">
         <v>74</v>
@@ -9140,21 +9384,21 @@
         <v>10</v>
       </c>
       <c r="E298" s="1" t="s">
-        <v>332</v>
+        <v>398</v>
       </c>
       <c r="F298" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G298" s="1" t="s">
-        <v>13</v>
+      <c r="G298" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="299" spans="1:7">
       <c r="A299" s="1" t="s">
-        <v>389</v>
+        <v>399</v>
       </c>
       <c r="B299" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C299" s="1" t="s">
         <v>74</v>
@@ -9163,21 +9407,21 @@
         <v>10</v>
       </c>
       <c r="E299" s="1" t="s">
-        <v>332</v>
+        <v>390</v>
       </c>
       <c r="F299" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G299" s="1" t="s">
-        <v>13</v>
+      <c r="G299" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="300" spans="1:7">
       <c r="A300" s="1" t="s">
-        <v>390</v>
+        <v>400</v>
       </c>
       <c r="B300" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C300" s="1" t="s">
         <v>74</v>
@@ -9186,21 +9430,21 @@
         <v>10</v>
       </c>
       <c r="E300" s="1" t="s">
-        <v>332</v>
+        <v>401</v>
       </c>
       <c r="F300" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G300" s="1" t="s">
-        <v>13</v>
+      <c r="G300" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="301" spans="1:7">
       <c r="A301" s="1" t="s">
-        <v>391</v>
+        <v>402</v>
       </c>
       <c r="B301" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C301" s="1" t="s">
         <v>74</v>
@@ -9209,21 +9453,21 @@
         <v>10</v>
       </c>
       <c r="E301" s="1" t="s">
-        <v>332</v>
+        <v>403</v>
       </c>
       <c r="F301" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G301" s="1" t="s">
-        <v>13</v>
+      <c r="G301" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="302" spans="1:7">
       <c r="A302" s="1" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="B302" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C302" s="1" t="s">
         <v>74</v>
@@ -9232,21 +9476,21 @@
         <v>10</v>
       </c>
       <c r="E302" s="1" t="s">
-        <v>332</v>
+        <v>405</v>
       </c>
       <c r="F302" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G302" s="1" t="s">
-        <v>13</v>
+      <c r="G302" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="303" spans="1:7">
       <c r="A303" s="1" t="s">
-        <v>393</v>
+        <v>406</v>
       </c>
       <c r="B303" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C303" s="1" t="s">
         <v>74</v>
@@ -9255,21 +9499,21 @@
         <v>10</v>
       </c>
       <c r="E303" s="1" t="s">
-        <v>332</v>
+        <v>407</v>
       </c>
       <c r="F303" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G303" s="1" t="s">
-        <v>13</v>
+      <c r="G303" s="4" t="s">
+        <v>361</v>
       </c>
     </row>
     <row r="304" spans="1:7">
       <c r="A304" s="1" t="s">
-        <v>394</v>
+        <v>408</v>
       </c>
       <c r="B304" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C304" s="1" t="s">
         <v>74</v>
@@ -9278,21 +9522,21 @@
         <v>10</v>
       </c>
       <c r="E304" s="1" t="s">
-        <v>332</v>
+        <v>409</v>
       </c>
       <c r="F304" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G304" s="1" t="s">
-        <v>13</v>
+      <c r="G304" s="4" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="305" spans="1:7">
       <c r="A305" s="1" t="s">
-        <v>395</v>
+        <v>411</v>
       </c>
       <c r="B305" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C305" s="1" t="s">
         <v>74</v>
@@ -9301,21 +9545,21 @@
         <v>10</v>
       </c>
       <c r="E305" s="1" t="s">
-        <v>332</v>
+        <v>363</v>
       </c>
       <c r="F305" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G305" s="1" t="s">
-        <v>13</v>
+      <c r="G305" s="4" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="306" spans="1:7">
       <c r="A306" s="1" t="s">
-        <v>396</v>
+        <v>412</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>334</v>
+        <v>358</v>
       </c>
       <c r="C306" s="1" t="s">
         <v>74</v>
@@ -9324,416 +9568,1382 @@
         <v>10</v>
       </c>
       <c r="E306" s="1" t="s">
-        <v>332</v>
+        <v>413</v>
       </c>
       <c r="F306" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="G306" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="307" hidden="1" spans="1:7">
-      <c r="A307" s="4" t="s">
-        <v>397</v>
-      </c>
-      <c r="B307" s="5" t="s">
-        <v>398</v>
-      </c>
-      <c r="C307" s="4" t="s">
-        <v>399</v>
-      </c>
-      <c r="D307" s="6" t="s">
+      <c r="G306" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="307" spans="1:7">
+      <c r="A307" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B307" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C307" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D307" s="1" t="s">
         <v>10</v>
       </c>
       <c r="E307" s="1" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="F307" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G307" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="308" hidden="1" spans="1:7">
+        <v>360</v>
+      </c>
+      <c r="G307" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="308" spans="1:7">
       <c r="A308" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="B308" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="B308" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C308" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D308" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E308" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="F308" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G308" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="309" spans="1:7">
+      <c r="A309" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="B309" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C309" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D309" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E309" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="F309" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G309" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="310" spans="1:7">
+      <c r="A310" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="B310" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C310" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D310" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E310" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="F310" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G310" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="311" spans="1:7">
+      <c r="A311" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="B311" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C311" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D311" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E311" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="F311" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G311" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="312" spans="1:7">
+      <c r="A312" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B312" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C312" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D312" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E312" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="F312" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G312" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="313" spans="1:7">
+      <c r="A313" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="B313" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C313" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D313" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E313" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="F313" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G313" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="314" spans="1:7">
+      <c r="A314" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="B314" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C314" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D314" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E314" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="F314" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G314" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="315" spans="1:7">
+      <c r="A315" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B315" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C315" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D315" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E315" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="F315" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G315" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="316" spans="1:7">
+      <c r="A316" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C316" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D316" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E316" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="F316" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G316" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="317" spans="1:7">
+      <c r="A317" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="B317" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C317" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D317" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E317" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="F317" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G317" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="318" spans="1:7">
+      <c r="A318" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="B318" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C318" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D318" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E318" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="F318" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G318" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="319" spans="1:7">
+      <c r="A319" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="B319" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C319" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D319" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E319" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="F319" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G319" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="320" spans="1:7">
+      <c r="A320" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="B320" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C320" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D320" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E320" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="F320" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G320" s="4" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="321" spans="1:7">
+      <c r="A321" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B321" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C321" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D321" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E321" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="F321" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G321" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="322" spans="1:7">
+      <c r="A322" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="B322" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C322" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D322" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E322" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="F322" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G322" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="323" spans="1:7">
+      <c r="A323" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B323" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C323" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D323" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E323" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="F323" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G323" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="324" spans="1:7">
+      <c r="A324" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="B324" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C324" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D324" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E324" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="F324" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G324" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="325" spans="1:7">
+      <c r="A325" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="B325" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C325" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D325" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E325" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="F325" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G325" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="326" spans="1:7">
+      <c r="A326" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B326" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C326" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D326" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E326" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="F326" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G326" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="327" spans="1:7">
+      <c r="A327" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B327" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C327" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D327" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E327" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="F327" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G327" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="328" spans="1:7">
+      <c r="A328" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="B328" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C328" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D328" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E328" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="F328" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G328" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="329" spans="1:7">
+      <c r="A329" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="B329" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C329" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D329" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E329" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="F329" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G329" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="330" spans="1:7">
+      <c r="A330" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="B330" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C330" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D330" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E330" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="F330" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G330" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="331" spans="1:7">
+      <c r="A331" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="B331" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C331" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D331" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E331" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F331" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G331" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="332" spans="1:7">
+      <c r="A332" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B332" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C332" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D332" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E332" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F332" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G332" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="333" spans="1:7">
+      <c r="A333" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="B333" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C333" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D333" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E333" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F333" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G333" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="334" spans="1:7">
+      <c r="A334" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="B334" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C334" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D334" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E334" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F334" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G334" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="335" spans="1:7">
+      <c r="A335" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="B335" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C335" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D335" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E335" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F335" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G335" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="336" spans="1:7">
+      <c r="A336" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B336" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C336" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D336" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E336" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F336" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G336" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="337" spans="1:7">
+      <c r="A337" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="B337" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C337" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D337" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E337" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F337" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G337" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="338" spans="1:7">
+      <c r="A338" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C338" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D338" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E338" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F338" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G338" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="339" spans="1:7">
+      <c r="A339" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="B339" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C339" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D339" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E339" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F339" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G339" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="340" spans="1:7">
+      <c r="A340" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B340" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C340" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D340" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E340" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F340" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G340" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="341" spans="1:7">
+      <c r="A341" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="B341" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C341" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D341" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E341" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F341" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G341" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="342" spans="1:7">
+      <c r="A342" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B342" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C342" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D342" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E342" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F342" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G342" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="343" spans="1:7">
+      <c r="A343" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B343" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C343" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D343" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E343" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F343" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G343" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="344" spans="1:7">
+      <c r="A344" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="B344" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C344" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D344" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E344" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F344" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G344" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="345" spans="1:7">
+      <c r="A345" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B345" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C345" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D345" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E345" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F345" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G345" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="346" spans="1:7">
+      <c r="A346" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B346" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C346" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D346" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E346" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F346" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G346" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="347" spans="1:7">
+      <c r="A347" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="B347" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C347" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D347" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E347" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F347" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G347" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="348" spans="1:7">
+      <c r="A348" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B348" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C348" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D348" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E348" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F348" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G348" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="349" hidden="1" spans="1:7">
+      <c r="A349" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B349" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="C349" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="D349" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E349" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="F349" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G349" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="350" hidden="1" spans="1:7">
+      <c r="A350" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B350" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="C308" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D308" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E308" s="1" t="s">
+      <c r="C350" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D350" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E350" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="F308" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G308" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="309" hidden="1" spans="1:7">
-      <c r="A309" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="B309" s="1" t="s">
+      <c r="F350" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G350" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="351" hidden="1" spans="1:7">
+      <c r="A351" s="1" t="s">
+        <v>482</v>
+      </c>
+      <c r="B351" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C309" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D309" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E309" s="1" t="s">
+      <c r="C351" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D351" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E351" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="F309" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G309" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="310" hidden="1" spans="1:7">
-      <c r="A310" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="B310" s="1" t="s">
+      <c r="F351" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G351" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="352" hidden="1" spans="1:7">
+      <c r="A352" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="B352" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C310" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D310" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E310" s="1" t="s">
+      <c r="C352" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D352" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E352" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="F310" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G310" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="311" hidden="1" spans="1:7">
-      <c r="A311" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="B311" s="1" t="s">
+      <c r="F352" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G352" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="353" hidden="1" spans="1:7">
+      <c r="A353" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B353" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C311" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D311" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E311" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="F311" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G311" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="312" hidden="1" spans="1:7">
-      <c r="A312" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="B312" s="1" t="s">
+      <c r="C353" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D353" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E353" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="F353" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G353" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="354" hidden="1" spans="1:7">
+      <c r="A354" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B354" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C312" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D312" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E312" s="1" t="s">
+      <c r="C354" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D354" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E354" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="F312" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G312" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="313" hidden="1" spans="1:7">
-      <c r="A313" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="B313" s="1" t="s">
+      <c r="F354" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G354" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="355" hidden="1" spans="1:7">
+      <c r="A355" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="B355" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C313" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D313" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E313" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="F313" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G313" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="314" hidden="1" spans="1:7">
-      <c r="A314" s="1" t="s">
-        <v>410</v>
-      </c>
-      <c r="B314" s="1" t="s">
+      <c r="C355" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D355" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E355" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="F355" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G355" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="356" hidden="1" spans="1:7">
+      <c r="A356" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B356" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C314" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D314" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E314" s="1" t="s">
+      <c r="C356" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D356" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E356" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="F314" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G314" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="315" hidden="1" spans="1:7">
-      <c r="A315" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="B315" s="1" t="s">
+      <c r="F356" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G356" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="357" hidden="1" spans="1:7">
+      <c r="A357" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="B357" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C315" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D315" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E315" s="1" t="s">
+      <c r="C357" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D357" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E357" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="F315" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G315" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="316" hidden="1" spans="1:7">
-      <c r="A316" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="B316" s="1" t="s">
+      <c r="F357" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G357" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="358" hidden="1" spans="1:7">
+      <c r="A358" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="B358" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C316" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D316" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E316" s="1" t="s">
+      <c r="C358" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D358" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E358" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F316" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G316" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="317" hidden="1" spans="1:7">
-      <c r="A317" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="B317" s="1" t="s">
+      <c r="F358" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G358" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="359" hidden="1" spans="1:7">
+      <c r="A359" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="B359" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C317" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D317" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E317" s="1" t="s">
+      <c r="C359" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D359" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E359" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F317" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G317" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="318" hidden="1" spans="1:7">
-      <c r="A318" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="B318" s="1" t="s">
+      <c r="F359" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G359" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="360" hidden="1" spans="1:7">
+      <c r="A360" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B360" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C318" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D318" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E318" s="1" t="s">
+      <c r="C360" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D360" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E360" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F318" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G318" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="319" hidden="1" spans="1:7">
-      <c r="A319" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="B319" s="1" t="s">
+      <c r="F360" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G360" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="361" hidden="1" spans="1:7">
+      <c r="A361" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="B361" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C319" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D319" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E319" s="1" t="s">
+      <c r="C361" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D361" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E361" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F319" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G319" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="320" hidden="1" spans="1:7">
-      <c r="A320" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="B320" s="1" t="s">
+      <c r="F361" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G361" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="362" hidden="1" spans="1:7">
+      <c r="A362" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B362" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C320" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D320" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E320" s="1" t="s">
+      <c r="C362" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D362" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E362" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F320" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G320" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="321" hidden="1" spans="1:7">
-      <c r="A321" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="B321" s="1" t="s">
+      <c r="F362" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G362" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="363" hidden="1" spans="1:7">
+      <c r="A363" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="B363" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C321" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D321" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E321" s="1" t="s">
+      <c r="C363" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D363" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E363" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F321" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G321" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="322" hidden="1" spans="1:7">
-      <c r="A322" s="1" t="s">
-        <v>418</v>
-      </c>
-      <c r="B322" s="1" t="s">
+      <c r="F363" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G363" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="364" hidden="1" spans="1:7">
+      <c r="A364" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B364" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C322" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D322" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E322" s="1" t="s">
+      <c r="C364" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D364" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E364" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F322" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G322" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="323" hidden="1" spans="1:7">
-      <c r="A323" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="B323" s="1" t="s">
+      <c r="F364" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G364" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="365" hidden="1" spans="1:7">
+      <c r="A365" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="B365" s="1" t="s">
         <v>258</v>
       </c>
-      <c r="C323" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="D323" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E323" s="1" t="s">
+      <c r="C365" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="D365" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E365" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="F323" s="1" t="s">
-        <v>401</v>
-      </c>
-      <c r="G323" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="324" spans="1:7">
-      <c r="F324" s="7"/>
-      <c r="G324" s="6"/>
+      <c r="F365" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="G365" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="366" spans="1:7">
+      <c r="F366" s="8"/>
+      <c r="G366" s="7"/>
     </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G323" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:G365" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="2">
-      <filters>
-        <filter val="scATAC"/>
-      </filters>
+      <customFilters>
+        <customFilter operator="equal" val="scATAC"/>
+      </customFilters>
     </filterColumn>
     <filterColumn colId="5">
       <filters>
@@ -9743,11 +10953,11 @@
     <extLst/>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="A281" r:id="rId1" display="GSM8671456"/>
-    <hyperlink ref="A294" r:id="rId2" display="GSM5737286"/>
-    <hyperlink ref="B307" r:id="rId3" display="https://www.10xgenomics.com/jp/datasets/pbmc-from-a-healthy-donor-no-cell-sorting-10-k-1-standard-2-0-0?utm_source=chatgpt.com"/>
-    <hyperlink ref="A311" r:id="rId4" display="GSM6611366" tooltip="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM6611366"/>
-    <hyperlink ref="A308" r:id="rId5" display="GSM6611363"/>
+    <hyperlink ref="A323" r:id="rId1" display="GSM8671456"/>
+    <hyperlink ref="A336" r:id="rId2" display="GSM5737286"/>
+    <hyperlink ref="B349" r:id="rId3" display="https://www.10xgenomics.com/jp/datasets/pbmc-from-a-healthy-donor-no-cell-sorting-10-k-1-standard-2-0-0?utm_source=chatgpt.com"/>
+    <hyperlink ref="A353" r:id="rId4" display="GSM6611366" tooltip="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSM6611366"/>
+    <hyperlink ref="A350" r:id="rId5" display="GSM6611363"/>
     <hyperlink ref="B2" r:id="rId6" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE149689"/>
     <hyperlink ref="B29" r:id="rId7" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE220188"/>
     <hyperlink ref="B124" r:id="rId8" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE222548"/>
@@ -9768,7 +10978,7 @@
     <hyperlink ref="B195" r:id="rId22" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE214546"/>
     <hyperlink ref="B243" r:id="rId22" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE214546"/>
     <hyperlink ref="B255" r:id="rId23" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE190992"/>
-    <hyperlink ref="B308" r:id="rId22" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE214546"/>
+    <hyperlink ref="B350" r:id="rId22" display="https://www.ncbi.nlm.nih.gov/geo/query/acc.cgi?acc=GSE214546"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>